<commit_message>
Chrome/Firefox version fields and an Excel software report per CI
The script now reads Chrome and Firefox (and falls back to the program list for
Edge). The new report lists, per Asset (CI), what was observed, the installed
software with versions, and a fleet view of program + version with machine
counts; engineers get only their own machines. Control characters from a PC
are stripped at intake because they crash the Excel export.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/templates/Software_Observation_Upload_Template.xlsx
+++ b/templates/Software_Observation_Upload_Template.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:W1"/>
+  <dimension ref="A1:Y1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -440,6 +440,8 @@
     <col width="22" customWidth="1" min="21" max="21"/>
     <col width="22" customWidth="1" min="22" max="22"/>
     <col width="22" customWidth="1" min="23" max="23"/>
+    <col width="22" customWidth="1" min="24" max="24"/>
+    <col width="22" customWidth="1" min="25" max="25"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -545,15 +547,25 @@
       </c>
       <c r="U1" t="inlineStr">
         <is>
-          <t>Browser version</t>
+          <t>Edge version</t>
         </is>
       </c>
       <c r="V1" t="inlineStr">
         <is>
+          <t>Chrome version</t>
+        </is>
+      </c>
+      <c r="W1" t="inlineStr">
+        <is>
+          <t>Firefox version</t>
+        </is>
+      </c>
+      <c r="X1" t="inlineStr">
+        <is>
           <t>Local administrators</t>
         </is>
       </c>
-      <c r="W1" t="inlineStr">
+      <c r="Y1" t="inlineStr">
         <is>
           <t>Remarks</t>
         </is>

</xml_diff>